<commit_message>
feat(empresas): importar CNAE principal opcional
</commit_message>
<xml_diff>
--- a/public/modelo-empresas.xlsx
+++ b/public/modelo-empresas.xlsx
@@ -44,8 +44,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H2"/>
   <cols>
-    <col min="1" max="7" width="22" style="1" customWidth="1"/>
+    <col min="1" max="8" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -82,6 +83,11 @@
       <c r="G1" s="2" t="inlineStr">
         <is>
           <t>cep</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>cnae_principal</t>
         </is>
       </c>
     </row>
@@ -121,6 +127,11 @@
           <t>01310100</t>
         </is>
       </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>4742300</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat(empresas): importar CNAE principal opcional (#27)
</commit_message>
<xml_diff>
--- a/public/modelo-empresas.xlsx
+++ b/public/modelo-empresas.xlsx
@@ -44,8 +44,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H2"/>
   <cols>
-    <col min="1" max="7" width="22" style="1" customWidth="1"/>
+    <col min="1" max="8" width="22" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -82,6 +83,11 @@
       <c r="G1" s="2" t="inlineStr">
         <is>
           <t>cep</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>cnae_principal</t>
         </is>
       </c>
     </row>
@@ -121,6 +127,11 @@
           <t>01310100</t>
         </is>
       </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>4742300</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>